<commit_message>
Remove unspecified original J value column from catalogue
</commit_message>
<xml_diff>
--- a/range-deliverables/final-canva-update/Fabric_Style_Dashboard_Final.xlsx
+++ b/range-deliverables/final-canva-update/Fabric_Style_Dashboard_Final.xlsx
@@ -9,9 +9,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Style Catalog" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Style Catalog'!$A$1:$J$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Style Catalog'!$A$1:$I$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Style Catalog'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Style Catalog'!$A$1:$J$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Style Catalog'!$A$1:$I$45</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -244,11 +244,6 @@
         <t>Names match the labelled PDF and Canva-importable presentation. Embedded shade names are retained where present. Other names describe visible colours, not verified supplier shade codes.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Original values retained for existing mapped rows. Extra colourways have blank values because no revised quantity or unit was supplied.</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -1673,7 +1668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1685,7 +1680,6 @@
     <col width="69" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1731,11 +1725,6 @@
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
-          <t>Original J Value (unit unspecified)</t>
-        </is>
-      </c>
-      <c r="J1" s="8" t="inlineStr">
-        <is>
           <t>Fit</t>
         </is>
       </c>
@@ -1777,10 +1766,7 @@
         </is>
       </c>
       <c r="H2" s="9" t="n"/>
-      <c r="I2" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J2" s="9" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -1823,10 +1809,7 @@
         </is>
       </c>
       <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J3" s="10" t="inlineStr">
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -1869,10 +1852,7 @@
         </is>
       </c>
       <c r="H4" s="9" t="n"/>
-      <c r="I4" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -1915,10 +1895,7 @@
         </is>
       </c>
       <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -1961,10 +1938,7 @@
         </is>
       </c>
       <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>Relaxed Fit</t>
         </is>
@@ -2007,10 +1981,7 @@
         </is>
       </c>
       <c r="H7" s="10" t="n"/>
-      <c r="I7" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>Relaxed Fit</t>
         </is>
@@ -2053,10 +2024,7 @@
         </is>
       </c>
       <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2099,10 +2067,7 @@
         </is>
       </c>
       <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2145,10 +2110,7 @@
         </is>
       </c>
       <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J10" s="9" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2191,10 +2153,7 @@
         </is>
       </c>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
+      <c r="I11" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2237,10 +2196,7 @@
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J12" s="9" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2283,10 +2239,7 @@
         </is>
       </c>
       <c r="H13" s="10" t="n"/>
-      <c r="I13" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2329,8 +2282,7 @@
         </is>
       </c>
       <c r="H14" s="9" t="n"/>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="9" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2373,8 +2325,7 @@
         </is>
       </c>
       <c r="H15" s="10" t="n"/>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="10" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2417,8 +2368,7 @@
         </is>
       </c>
       <c r="H16" s="9" t="n"/>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="9" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2461,8 +2411,7 @@
         </is>
       </c>
       <c r="H17" s="10" t="n"/>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="10" t="inlineStr">
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2505,8 +2454,7 @@
         </is>
       </c>
       <c r="H18" s="9" t="n"/>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="9" t="inlineStr">
+      <c r="I18" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2549,8 +2497,7 @@
         </is>
       </c>
       <c r="H19" s="10" t="n"/>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="10" t="inlineStr">
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2593,8 +2540,7 @@
         </is>
       </c>
       <c r="H20" s="9" t="n"/>
-      <c r="I20" s="11" t="n"/>
-      <c r="J20" s="9" t="inlineStr">
+      <c r="I20" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2637,8 +2583,7 @@
         </is>
       </c>
       <c r="H21" s="10" t="n"/>
-      <c r="I21" s="11" t="n"/>
-      <c r="J21" s="10" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2681,10 +2626,7 @@
         </is>
       </c>
       <c r="H22" s="9" t="n"/>
-      <c r="I22" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J22" s="9" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2727,10 +2669,7 @@
         </is>
       </c>
       <c r="H23" s="10" t="n"/>
-      <c r="I23" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J23" s="10" t="inlineStr">
+      <c r="I23" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2773,10 +2712,7 @@
         </is>
       </c>
       <c r="H24" s="9" t="n"/>
-      <c r="I24" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J24" s="9" t="inlineStr">
+      <c r="I24" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2819,10 +2755,7 @@
         </is>
       </c>
       <c r="H25" s="10" t="n"/>
-      <c r="I25" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J25" s="10" t="inlineStr">
+      <c r="I25" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2865,10 +2798,7 @@
         </is>
       </c>
       <c r="H26" s="9" t="n"/>
-      <c r="I26" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J26" s="9" t="inlineStr">
+      <c r="I26" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2911,10 +2841,7 @@
         </is>
       </c>
       <c r="H27" s="10" t="n"/>
-      <c r="I27" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J27" s="10" t="inlineStr">
+      <c r="I27" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2957,8 +2884,7 @@
         </is>
       </c>
       <c r="H28" s="9" t="n"/>
-      <c r="I28" s="11" t="n"/>
-      <c r="J28" s="9" t="inlineStr">
+      <c r="I28" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3001,10 +2927,7 @@
         </is>
       </c>
       <c r="H29" s="10" t="n"/>
-      <c r="I29" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J29" s="10" t="inlineStr">
+      <c r="I29" s="10" t="inlineStr">
         <is>
           <t>Relaxed Fit</t>
         </is>
@@ -3047,10 +2970,7 @@
         </is>
       </c>
       <c r="H30" s="9" t="n"/>
-      <c r="I30" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J30" s="9" t="inlineStr">
+      <c r="I30" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3093,10 +3013,7 @@
         </is>
       </c>
       <c r="H31" s="10" t="n"/>
-      <c r="I31" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J31" s="10" t="inlineStr">
+      <c r="I31" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3139,10 +3056,7 @@
         </is>
       </c>
       <c r="H32" s="9" t="n"/>
-      <c r="I32" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J32" s="9" t="inlineStr">
+      <c r="I32" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3185,10 +3099,7 @@
         </is>
       </c>
       <c r="H33" s="10" t="n"/>
-      <c r="I33" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J33" s="10" t="inlineStr">
+      <c r="I33" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3231,10 +3142,7 @@
         </is>
       </c>
       <c r="H34" s="9" t="n"/>
-      <c r="I34" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J34" s="9" t="inlineStr">
+      <c r="I34" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3277,10 +3185,7 @@
         </is>
       </c>
       <c r="H35" s="10" t="n"/>
-      <c r="I35" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J35" s="10" t="inlineStr">
+      <c r="I35" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3323,10 +3228,7 @@
         </is>
       </c>
       <c r="H36" s="9" t="n"/>
-      <c r="I36" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J36" s="9" t="inlineStr">
+      <c r="I36" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3369,10 +3271,7 @@
         </is>
       </c>
       <c r="H37" s="10" t="n"/>
-      <c r="I37" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J37" s="10" t="inlineStr">
+      <c r="I37" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3415,10 +3314,7 @@
         </is>
       </c>
       <c r="H38" s="9" t="n"/>
-      <c r="I38" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J38" s="9" t="inlineStr">
+      <c r="I38" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3461,10 +3357,7 @@
         </is>
       </c>
       <c r="H39" s="10" t="n"/>
-      <c r="I39" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J39" s="10" t="inlineStr">
+      <c r="I39" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3507,10 +3400,7 @@
         </is>
       </c>
       <c r="H40" s="9" t="n"/>
-      <c r="I40" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J40" s="9" t="inlineStr">
+      <c r="I40" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3553,10 +3443,7 @@
         </is>
       </c>
       <c r="H41" s="10" t="n"/>
-      <c r="I41" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J41" s="10" t="inlineStr">
+      <c r="I41" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3599,10 +3486,7 @@
         </is>
       </c>
       <c r="H42" s="9" t="n"/>
-      <c r="I42" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J42" s="9" t="inlineStr">
+      <c r="I42" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3645,10 +3529,7 @@
         </is>
       </c>
       <c r="H43" s="10" t="n"/>
-      <c r="I43" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J43" s="10" t="inlineStr">
+      <c r="I43" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3691,10 +3572,7 @@
         </is>
       </c>
       <c r="H44" s="9" t="n"/>
-      <c r="I44" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="J44" s="9" t="inlineStr">
+      <c r="I44" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3737,17 +3615,14 @@
         </is>
       </c>
       <c r="H45" s="10" t="n"/>
-      <c r="I45" s="10" t="n">
-        <v>400</v>
-      </c>
-      <c r="J45" s="10" t="inlineStr">
+      <c r="I45" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J45"/>
+  <autoFilter ref="A1:I45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Add quantity of 400 for every final colourway
</commit_message>
<xml_diff>
--- a/range-deliverables/final-canva-update/Fabric_Style_Dashboard_Final.xlsx
+++ b/range-deliverables/final-canva-update/Fabric_Style_Dashboard_Final.xlsx
@@ -9,9 +9,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Style Catalog" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Style Catalog'!$A$1:$I$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Style Catalog'!$A$1:$J$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Style Catalog'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Style Catalog'!$A$1:$I$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Style Catalog'!$A$1:$J$45</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -155,6 +155,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1668,7 +1674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1679,7 +1685,8 @@
     <col width="38" customWidth="1" min="6" max="6"/>
     <col width="69" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1725,6 +1732,11 @@
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
           <t>Fit</t>
         </is>
       </c>
@@ -1766,7 +1778,10 @@
         </is>
       </c>
       <c r="H2" s="9" t="n"/>
-      <c r="I2" s="9" t="inlineStr">
+      <c r="I2" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -1809,7 +1824,10 @@
         </is>
       </c>
       <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="I3" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -1852,7 +1870,10 @@
         </is>
       </c>
       <c r="H4" s="9" t="n"/>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -1895,7 +1916,10 @@
         </is>
       </c>
       <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="inlineStr">
+      <c r="I5" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -1938,7 +1962,10 @@
         </is>
       </c>
       <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="I6" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>Relaxed Fit</t>
         </is>
@@ -1981,7 +2008,10 @@
         </is>
       </c>
       <c r="H7" s="10" t="n"/>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="I7" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
         <is>
           <t>Relaxed Fit</t>
         </is>
@@ -2024,7 +2054,10 @@
         </is>
       </c>
       <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I8" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2067,7 +2100,10 @@
         </is>
       </c>
       <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I9" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2110,7 +2146,10 @@
         </is>
       </c>
       <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="inlineStr">
+      <c r="I10" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2153,7 +2192,10 @@
         </is>
       </c>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="inlineStr">
+      <c r="I11" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2196,7 +2238,10 @@
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="inlineStr">
+      <c r="I12" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2239,7 +2284,10 @@
         </is>
       </c>
       <c r="H13" s="10" t="n"/>
-      <c r="I13" s="10" t="inlineStr">
+      <c r="I13" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2282,7 +2330,10 @@
         </is>
       </c>
       <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="I14" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2325,7 +2376,10 @@
         </is>
       </c>
       <c r="H15" s="10" t="n"/>
-      <c r="I15" s="10" t="inlineStr">
+      <c r="I15" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2368,7 +2422,10 @@
         </is>
       </c>
       <c r="H16" s="9" t="n"/>
-      <c r="I16" s="9" t="inlineStr">
+      <c r="I16" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2411,7 +2468,10 @@
         </is>
       </c>
       <c r="H17" s="10" t="n"/>
-      <c r="I17" s="10" t="inlineStr">
+      <c r="I17" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2454,7 +2514,10 @@
         </is>
       </c>
       <c r="H18" s="9" t="n"/>
-      <c r="I18" s="9" t="inlineStr">
+      <c r="I18" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2497,7 +2560,10 @@
         </is>
       </c>
       <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="inlineStr">
+      <c r="I19" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2540,7 +2606,10 @@
         </is>
       </c>
       <c r="H20" s="9" t="n"/>
-      <c r="I20" s="9" t="inlineStr">
+      <c r="I20" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2583,7 +2652,10 @@
         </is>
       </c>
       <c r="H21" s="10" t="n"/>
-      <c r="I21" s="10" t="inlineStr">
+      <c r="I21" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2626,7 +2698,10 @@
         </is>
       </c>
       <c r="H22" s="9" t="n"/>
-      <c r="I22" s="9" t="inlineStr">
+      <c r="I22" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2669,7 +2744,10 @@
         </is>
       </c>
       <c r="H23" s="10" t="n"/>
-      <c r="I23" s="10" t="inlineStr">
+      <c r="I23" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2712,7 +2790,10 @@
         </is>
       </c>
       <c r="H24" s="9" t="n"/>
-      <c r="I24" s="9" t="inlineStr">
+      <c r="I24" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2755,7 +2836,10 @@
         </is>
       </c>
       <c r="H25" s="10" t="n"/>
-      <c r="I25" s="10" t="inlineStr">
+      <c r="I25" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2798,7 +2882,10 @@
         </is>
       </c>
       <c r="H26" s="9" t="n"/>
-      <c r="I26" s="9" t="inlineStr">
+      <c r="I26" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2841,7 +2928,10 @@
         </is>
       </c>
       <c r="H27" s="10" t="n"/>
-      <c r="I27" s="10" t="inlineStr">
+      <c r="I27" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2884,7 +2974,10 @@
         </is>
       </c>
       <c r="H28" s="9" t="n"/>
-      <c r="I28" s="9" t="inlineStr">
+      <c r="I28" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -2927,7 +3020,10 @@
         </is>
       </c>
       <c r="H29" s="10" t="n"/>
-      <c r="I29" s="10" t="inlineStr">
+      <c r="I29" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
         <is>
           <t>Relaxed Fit</t>
         </is>
@@ -2970,7 +3066,10 @@
         </is>
       </c>
       <c r="H30" s="9" t="n"/>
-      <c r="I30" s="9" t="inlineStr">
+      <c r="I30" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3013,7 +3112,10 @@
         </is>
       </c>
       <c r="H31" s="10" t="n"/>
-      <c r="I31" s="10" t="inlineStr">
+      <c r="I31" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J31" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3056,7 +3158,10 @@
         </is>
       </c>
       <c r="H32" s="9" t="n"/>
-      <c r="I32" s="9" t="inlineStr">
+      <c r="I32" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3099,7 +3204,10 @@
         </is>
       </c>
       <c r="H33" s="10" t="n"/>
-      <c r="I33" s="10" t="inlineStr">
+      <c r="I33" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J33" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3142,7 +3250,10 @@
         </is>
       </c>
       <c r="H34" s="9" t="n"/>
-      <c r="I34" s="9" t="inlineStr">
+      <c r="I34" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J34" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3185,7 +3296,10 @@
         </is>
       </c>
       <c r="H35" s="10" t="n"/>
-      <c r="I35" s="10" t="inlineStr">
+      <c r="I35" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J35" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3228,7 +3342,10 @@
         </is>
       </c>
       <c r="H36" s="9" t="n"/>
-      <c r="I36" s="9" t="inlineStr">
+      <c r="I36" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J36" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3271,7 +3388,10 @@
         </is>
       </c>
       <c r="H37" s="10" t="n"/>
-      <c r="I37" s="10" t="inlineStr">
+      <c r="I37" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J37" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3314,7 +3434,10 @@
         </is>
       </c>
       <c r="H38" s="9" t="n"/>
-      <c r="I38" s="9" t="inlineStr">
+      <c r="I38" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3357,7 +3480,10 @@
         </is>
       </c>
       <c r="H39" s="10" t="n"/>
-      <c r="I39" s="10" t="inlineStr">
+      <c r="I39" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J39" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3400,7 +3526,10 @@
         </is>
       </c>
       <c r="H40" s="9" t="n"/>
-      <c r="I40" s="9" t="inlineStr">
+      <c r="I40" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J40" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3443,7 +3572,10 @@
         </is>
       </c>
       <c r="H41" s="10" t="n"/>
-      <c r="I41" s="10" t="inlineStr">
+      <c r="I41" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J41" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3486,7 +3618,10 @@
         </is>
       </c>
       <c r="H42" s="9" t="n"/>
-      <c r="I42" s="9" t="inlineStr">
+      <c r="I42" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J42" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3529,7 +3664,10 @@
         </is>
       </c>
       <c r="H43" s="10" t="n"/>
-      <c r="I43" s="10" t="inlineStr">
+      <c r="I43" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J43" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3572,7 +3710,10 @@
         </is>
       </c>
       <c r="H44" s="9" t="n"/>
-      <c r="I44" s="9" t="inlineStr">
+      <c r="I44" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J44" s="9" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
@@ -3615,14 +3756,17 @@
         </is>
       </c>
       <c r="H45" s="10" t="n"/>
-      <c r="I45" s="10" t="inlineStr">
+      <c r="I45" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="J45" s="10" t="inlineStr">
         <is>
           <t>Slim Fit</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I45"/>
+  <autoFilter ref="A1:J45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Add part-specific Pantone TCX references with source and proposed status
</commit_message>
<xml_diff>
--- a/range-deliverables/final-canva-update/Fabric_Style_Dashboard_Final.xlsx
+++ b/range-deliverables/final-canva-update/Fabric_Style_Dashboard_Final.xlsx
@@ -9,9 +9,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Style Catalog" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Style Catalog'!$A$1:$J$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Style Catalog'!$A$1:$K$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Style Catalog'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Style Catalog'!$A$1:$J$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Style Catalog'!$A$1:$K$45</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -55,6 +55,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="00243B43"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="8">
@@ -124,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -161,6 +166,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -243,11 +257,239 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Range update</author>
+    <author>Pantone reference methodology</author>
   </authors>
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>Names match the labelled PDF and Canva-importable presentation. Embedded shade names are retained where present. Other names describe visible colours, not verified supplier shade codes.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K2" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K3" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K4" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K6" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K7" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.
+SOURCE LABEL ISSUE: The supplied PDF prints 19-0223 TCX for Eucalyptus. That code was not found in the checked reference dataset. Proposed 16-0110 TCX Desert Sage follows the visible grey-green render. This is NOT official Pantone Eucalyptus (15-0513); the marketing colour name is retained. Confirm with supplier / physical TCX standard.</t>
+      </text>
+    </comment>
+    <comment ref="K8" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.
+SOURCE LABEL ISSUE: The supplied PDF appears to print 19-2421 TCX for Earthy Brown. That code was not found in the checked reference dataset. Proposed 18-1222 TCX Cocoa Brown follows the brown render. Confirm the intended source code with supplier / physical TCX standard.</t>
+      </text>
+    </comment>
+    <comment ref="K9" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K10" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K11" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K12" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K13" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K14" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K15" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K16" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K17" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K18" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K19" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K20" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K21" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K22" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K23" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K24" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K25" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K26" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K27" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K28" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K29" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K30" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K31" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K32" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K33" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K34" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K35" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K36" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K37" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K38" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K39" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K40" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K41" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K42" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K43" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K44" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+      </text>
+    </comment>
+    <comment ref="K45" authorId="1" shapeId="0">
+      <text>
+        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
       </text>
     </comment>
   </commentList>
@@ -1674,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1687,6 +1929,7 @@
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="100" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1740,6 +1983,11 @@
           <t>Fit</t>
         </is>
       </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>Pantone TCX Reference</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="245" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -1786,6 +2034,13 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>Body / collar — Dark Olive: 19-0323 TCX (Chive) [PROPOSED]
+Side panel / contrast sleeve — Off White: 11-0602 TCX (Snow White) [PROPOSED]
+Cable stripe — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="245" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -1832,6 +2087,13 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>Body / collar — Denim Blue: 17-4021 TCX (Faded Denim) [PROPOSED]
+Side panel / contrast sleeve — Off White: 11-0602 TCX (Snow White) [PROPOSED]
+Cable stripe — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="245" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
@@ -1878,6 +2140,11 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Body / collar / rib trim — Classic Beige: 15-1217 TCX (Mojave Desert) [PDF]</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="245" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -1924,6 +2191,11 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Body / collar / rib trim — Grounded Green: 19-0323 TCX (Chive) [PDF]</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="245" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -1970,6 +2242,12 @@
           <t>Relaxed Fit</t>
         </is>
       </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>Ground — Classic Beige: 15-1217 TCX (Mojave Desert) [PDF]
+Floral motif — Bright White: 11-0601 TCX (Bright White) [PDF]</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="245" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -2016,6 +2294,13 @@
           <t>Relaxed Fit</t>
         </is>
       </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Ground — Eucalyptus: 16-0110 TCX (Desert Sage) [PROPOSED]
+Floral motif — Natural Cotton: 11-0602 TCX (Snow White) [PDF]
+SOURCE-CODE CHECK REQUIRED — see cell comment.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="245" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -2062,6 +2347,13 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>Body / collar — Earthy Brown: 18-1222 TCX (Cocoa Brown) [PROPOSED]
+Collar / placket / cuff piping — Natural Cotton: 11-0602 TCX (Snow White) [PDF]
+SOURCE-CODE CHECK REQUIRED — see cell comment.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="245" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -2108,6 +2400,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>Body / collar — Classic Navy: 19-4029 TCX (Navy Peony) [PDF]
+Collar / placket / cuff piping — Natural Cotton: 11-0602 TCX (Snow White) [PDF]</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="245" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
@@ -2154,6 +2452,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>Body — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Collar / placket stripes — Chocolate Brown: 19-0912 TCX (Chocolate Brown) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="245" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -2200,6 +2504,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>Body — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]
+Collar / placket stripes — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="245" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -2246,6 +2556,11 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="245" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -2292,6 +2607,11 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K13" s="15" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Black: 19-0303 TCX (Jet Black) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="245" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -2338,6 +2658,11 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="245" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -2384,6 +2709,11 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Sage Green: 16-0110 TCX (Desert Sage) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="245" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
@@ -2430,6 +2760,11 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Powder Blue: 14-4214 TCX (Powder Blue) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="245" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -2476,6 +2811,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K17" s="15" t="inlineStr">
+        <is>
+          <t>Body — Powder Blue: 14-4214 TCX (Powder Blue) [PROPOSED]
+Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="245" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -2522,6 +2863,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>Body — Dusty Rose: 14-1506 TCX (Rose Smoke) [PROPOSED]
+Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="245" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -2568,6 +2915,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K19" s="15" t="inlineStr">
+        <is>
+          <t>Body — Sage Green: 16-0110 TCX (Desert Sage) [PROPOSED]
+Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="245" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -2614,6 +2967,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K20" s="14" t="inlineStr">
+        <is>
+          <t>Body — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
+Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="245" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -2660,6 +3019,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K21" s="15" t="inlineStr">
+        <is>
+          <t>Body — Oatmeal: 13-0401 TCX (Oatmeal) [PROPOSED]
+Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="245" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
@@ -2706,6 +3071,13 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K22" s="14" t="inlineStr">
+        <is>
+          <t>Ground — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Chest panel / collar — Denim Blue: 17-4021 TCX (Faded Denim) [PROPOSED]
+Fine panel borders — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="245" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -2752,6 +3124,13 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K23" s="15" t="inlineStr">
+        <is>
+          <t>Ground — Butter Yellow: 13-0822 TCX (Sunlight) [PROPOSED]
+Chest panel / collar — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Fine panel borders — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="245" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
@@ -2798,6 +3177,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>Body / collar — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
+Collar / cuff tipping — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="245" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -2844,6 +3229,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K25" s="15" t="inlineStr">
+        <is>
+          <t>Body / collar — Rust: 18-1248 TCX (Rust) [PROPOSED]
+Collar / cuff tipping — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="245" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
@@ -2890,6 +3281,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K26" s="14" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Off White: 11-0602 TCX (Snow White) [PROPOSED]
+Horizontal stripes — Denim Blue: 17-4021 TCX (Faded Denim) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="245" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -2936,6 +3333,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K27" s="15" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Off White: 11-0602 TCX (Snow White) [PROPOSED]
+Horizontal stripes — Rust: 18-1248 TCX (Rust) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="245" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
@@ -2982,6 +3385,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K28" s="14" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Off White: 11-0602 TCX (Snow White) [PROPOSED]
+Horizontal stripes — Olive Green: 18-0622 TCX (Olive Drab) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="245" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
@@ -3028,6 +3437,14 @@
           <t>Relaxed Fit</t>
         </is>
       </c>
+      <c r="K29" s="15" t="inlineStr">
+        <is>
+          <t>Mesh ground — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Neck / shoulder stripes / back graphic — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]
+Badge dark details — Charcoal: 19-4007 TCX (Anthracite) [PROPOSED]
+Badge light details — White: 11-0601 TCX (Bright White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="245" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
@@ -3074,6 +3491,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K30" s="14" t="inlineStr">
+        <is>
+          <t>Ground / collar / rib trim — Powder Blue: 14-4214 TCX (Powder Blue) [PROPOSED]
+Vertical pinstripes — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="245" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
@@ -3120,6 +3543,13 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K31" s="15" t="inlineStr">
+        <is>
+          <t>Ground / collar / rib trim — White: 11-0601 TCX (Bright White) [PROPOSED]
+Primary vertical pinstripes — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
+Secondary vertical pinstripes — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="245" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
@@ -3166,6 +3596,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K32" s="14" t="inlineStr">
+        <is>
+          <t>Body — Deep Teal: 19-4914 TCX (Deep Teal) [PROPOSED]
+Collar / zip trim / tipping / stag — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="245" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
@@ -3212,6 +3648,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K33" s="15" t="inlineStr">
+        <is>
+          <t>Body — Sage Green: 16-0110 TCX (Desert Sage) [PROPOSED]
+Collar / zip trim / tipping / stag — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="245" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
@@ -3258,6 +3700,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K34" s="14" t="inlineStr">
+        <is>
+          <t>Ground / collar / cuffs — White: 11-0601 TCX (Bright White) [PROPOSED]
+Broad chest band — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
+Fine stripe borders — Powder Blue: 14-4214 TCX (Powder Blue) [PROPOSED]
+Badge / zip-pull accent — Red: 18-1664 TCX (Fiery Red) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="245" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
@@ -3304,6 +3754,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K35" s="15" t="inlineStr">
+        <is>
+          <t>Ground / collar / cuffs — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
+Broad chest band — Butter Yellow: 13-0822 TCX (Sunlight) [PROPOSED]
+Fine stripe borders — Dusty Pink: 14-1316 TCX (Dusty Pink) [PROPOSED]
+Badge / zip-pull accent — Red: 18-1664 TCX (Fiery Red) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="245" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
@@ -3350,6 +3808,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K36" s="14" t="inlineStr">
+        <is>
+          <t>Ground / collar / placket — Mustard Yellow: 14-0952 TCX (Spicy Mustard) [PROPOSED]
+Broad stripes — Royal Blue: 17-4041 TCX (Marina) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="245" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
@@ -3396,6 +3860,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K37" s="15" t="inlineStr">
+        <is>
+          <t>Ground — Emerald Green: 17-5641 TCX (Emerald) [PROPOSED]
+Collar / broad stripes — Purple: 19-3642 TCX (Royal Purple) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="245" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
@@ -3442,6 +3912,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K38" s="14" t="inlineStr">
+        <is>
+          <t>Ground / collar / rib trim — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Fine stripes / emblem — Taupe: 16-1105 TCX (Plaza Taupe) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="245" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
@@ -3488,8 +3964,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
-    </row>
-    <row r="40" ht="245" customHeight="1">
+      <c r="K39" s="15" t="inlineStr">
+        <is>
+          <t>Ground / collar — Royal Blue: 17-4041 TCX (Marina) [PROPOSED]
+Fine stripes / rib trim — White: 11-0601 TCX (Bright White) [PROPOSED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="265" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
           <t>ST-17-1</t>
@@ -3534,6 +4016,16 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K40" s="14" t="inlineStr">
+        <is>
+          <t>Body / collar — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Embroidery petals — White: 11-0601 TCX (Bright White) [PROPOSED]
+Embroidery leaves — Olive Green: 18-0622 TCX (Olive Drab) [PROPOSED]
+Embroidery stems / outlines — Chocolate Brown: 19-0912 TCX (Chocolate Brown) [PROPOSED]
+Flower centres / bee yellow — Mustard Yellow: 14-0952 TCX (Spicy Mustard) [PROPOSED]
+Bee dark details — Black: 19-0303 TCX (Jet Black) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="245" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
@@ -3580,6 +4072,15 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K41" s="15" t="inlineStr">
+        <is>
+          <t>Body / collar — Dark Olive: 19-0323 TCX (Chive) [PROPOSED]
+Embroidery petals / light outlines — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Embroidery leaves — Sage Green: 16-0110 TCX (Desert Sage) [PROPOSED]
+Flower centres / bee yellow — Mustard Yellow: 14-0952 TCX (Spicy Mustard) [PROPOSED]
+Bee dark details — Black: 19-0303 TCX (Jet Black) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="245" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
@@ -3626,6 +4127,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K42" s="14" t="inlineStr">
+        <is>
+          <t>Body / collar — Chocolate Brown: 19-0912 TCX (Chocolate Brown) [PROPOSED]
+Collar / cuff / hem tipping — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="245" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
@@ -3672,6 +4179,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K43" s="15" t="inlineStr">
+        <is>
+          <t>Body / collar — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Collar / cuff / hem tipping — Chocolate Brown: 19-0912 TCX (Chocolate Brown) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="245" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
@@ -3718,6 +4231,13 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K44" s="14" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
+Warm micro stripes — Taupe: 16-1105 TCX (Plaza Taupe) [PROPOSED]
+Cool micro stripes — Grey: 17-4402 TCX (Neutral Gray) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="245" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
@@ -3764,9 +4284,16 @@
           <t>Slim Fit</t>
         </is>
       </c>
+      <c r="K45" s="15" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]
+Warm micro stripes — Taupe: 16-1105 TCX (Plaza Taupe) [PROPOSED]
+Cool micro stripes — Grey: 17-4402 TCX (Neutral Gray) [PROPOSED]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J45"/>
+  <autoFilter ref="A1:K45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Replace colour-name guesses with image-sampled TCX proposals and visual comparisons
</commit_message>
<xml_diff>
--- a/range-deliverables/final-canva-update/Fabric_Style_Dashboard_Final.xlsx
+++ b/range-deliverables/final-canva-update/Fabric_Style_Dashboard_Final.xlsx
@@ -9,9 +9,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Style Catalog" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Style Catalog'!$A$1:$K$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Style Catalog'!$A$1:$M$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Style Catalog'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Style Catalog'!$A$1:$K$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Style Catalog'!$A$1:$M$45</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -59,6 +59,11 @@
     <font>
       <name val="Aptos"/>
       <color rgb="00243B43"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="0020313B"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -129,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -175,6 +180,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -257,7 +268,8 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Range update</author>
-    <author>Pantone reference methodology</author>
+    <author>Image-based Pantone methodology</author>
+    <author>Image inspection</author>
   </authors>
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -267,229 +279,389 @@
     </comment>
     <comment ref="K1" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.</t>
       </text>
     </comment>
-    <comment ref="K2" authorId="1" shapeId="0">
+    <comment ref="L1" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.</t>
       </text>
     </comment>
-    <comment ref="K3" authorId="1" shapeId="0">
+    <comment ref="M1" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.</t>
       </text>
     </comment>
-    <comment ref="K4" authorId="1" shapeId="0">
+    <comment ref="L2" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-01_01.jpg, pixel box (233, 401, 263, 445), selector median, 1320 selected pixels.
+Side panel / contrast sleeve: ST-01_01.jpg, pixel box (336, 419, 366, 463), selector median, 1320 selected pixels.
+Cable stripe: ST-01_01.jpg, pixel box (380, 401, 389, 463), selector dark, 113 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K5" authorId="1" shapeId="0">
+    <comment ref="L3" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-01_02.jpg, pixel box (216, 401, 245, 445), selector median, 1276 selected pixels.
+Side panel / contrast sleeve: ST-01_02.jpg, pixel box (342, 419, 372, 463), selector median, 1320 selected pixels.
+Cable stripe: ST-01_02.jpg, pixel box (387, 401, 397, 463), selector dark, 124 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K6" authorId="1" shapeId="0">
+    <comment ref="L4" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar / rib trim: ST-02_01.jpg, pixel box (342, 361, 373, 401), selector median, 1240 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K7" authorId="1" shapeId="0">
+    <comment ref="L5" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.
-SOURCE LABEL ISSUE: The supplied PDF prints 19-0223 TCX for Eucalyptus. That code was not found in the checked reference dataset. Proposed 16-0110 TCX Desert Sage follows the visible grey-green render. This is NOT official Pantone Eucalyptus (15-0513); the marketing colour name is retained. Confirm with supplier / physical TCX standard.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar / rib trim: ST-02_02.jpg, pixel box (342, 377, 373, 417), selector median, 1240 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K8" authorId="1" shapeId="0">
+    <comment ref="L6" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.
-SOURCE LABEL ISSUE: The supplied PDF appears to print 19-2421 TCX for Earthy Brown. That code was not found in the checked reference dataset. Proposed 18-1222 TCX Cocoa Brown follows the brown render. Confirm the intended source code with supplier / physical TCX standard.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground: ST-03_01.jpg, pixel box (180, 328, 316, 494), selector dark, 4516 selected pixels.
+Floral motif: ST-03_01.jpg, pixel box (180, 328, 316, 494), selector light, 4544 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K9" authorId="1" shapeId="0">
+    <comment ref="L7" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground: ST-03_02.jpg, pixel box (180, 328, 316, 494), selector dark, 4540 selected pixels.
+Floral motif: ST-03_02.jpg, pixel box (180, 328, 316, 494), selector light, 4580 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K10" authorId="1" shapeId="0">
+    <comment ref="L8" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-04_01.jpg, pixel box (342, 464, 373, 505), selector median, 1271 selected pixels.
+Collar / placket / cuff piping: ST-04_01.jpg, pixel box (321, 329, 337, 386), selector light, 183 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K11" authorId="1" shapeId="0">
+    <comment ref="L9" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-04_02.jpg, pixel box (342, 464, 373, 505), selector median, 1271 selected pixels.
+Collar / placket / cuff piping: ST-04_02.jpg, pixel box (321, 329, 337, 386), selector light, 183 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K12" authorId="1" shapeId="0">
+    <comment ref="L10" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-05_01.jpg, pixel box (159, 431, 183, 473), selector median, 1008 selected pixels.
+Collar / placket stripes: ST-05_01.jpg, pixel box (204, 291, 237, 366), selector dark, 498 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K13" authorId="1" shapeId="0">
+    <comment ref="L11" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-05_02.jpg, pixel box (160, 431, 183, 473), selector median, 966 selected pixels.
+Collar / placket stripes: ST-05_02.jpg, pixel box (205, 291, 237, 366), selector light, 488 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K14" authorId="1" shapeId="0">
+    <comment ref="L12" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / neck / cuffs / hem: ST-08_01.jpg, pixel box (141, 406, 157, 446), selector median, 640 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K15" authorId="1" shapeId="0">
+    <comment ref="L13" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / neck / cuffs / hem: ST-08_02.jpg, pixel box (141, 406, 158, 446), selector median, 680 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K16" authorId="1" shapeId="0">
+    <comment ref="L14" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / neck / cuffs / hem: ST-08_03.jpg, pixel box (141, 406, 157, 446), selector median, 640 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K17" authorId="1" shapeId="0">
+    <comment ref="L15" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / neck / cuffs / hem: ST-08_04.jpg, pixel box (141, 406, 157, 446), selector median, 640 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K18" authorId="1" shapeId="0">
+    <comment ref="L16" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / neck / cuffs / hem: ST-08_05.jpg, pixel box (141, 406, 157, 446), selector median, 640 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K19" authorId="1" shapeId="0">
+    <comment ref="L17" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-20_01.jpg, pixel box (116, 390, 132, 430), selector median, 640 selected pixels.
+Collar / placket / cuffs / hem: ST-20_01.jpg, pixel box (108, 568, 202, 593), selector light, 473 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K20" authorId="1" shapeId="0">
+    <comment ref="L18" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-20_02.jpg, pixel box (116, 390, 132, 430), selector median, 640 selected pixels.
+Collar / placket / cuffs / hem: ST-20_02.jpg, pixel box (108, 568, 202, 593), selector light, 484 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K21" authorId="1" shapeId="0">
+    <comment ref="L19" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-20_03.jpg, pixel box (116, 390, 132, 430), selector median, 640 selected pixels.
+Collar / placket / cuffs / hem: ST-20_03.jpg, pixel box (108, 568, 202, 593), selector light, 474 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K22" authorId="1" shapeId="0">
+    <comment ref="L20" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-20_04.jpg, pixel box (116, 390, 132, 430), selector median, 640 selected pixels.
+Collar / placket / cuffs / hem: ST-20_04.jpg, pixel box (108, 568, 202, 593), selector light, 474 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K23" authorId="1" shapeId="0">
+    <comment ref="L21" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-20_05.jpg, pixel box (116, 390, 133, 430), selector median, 680 selected pixels.
+Collar / placket / cuffs / hem: ST-20_05.jpg, pixel box (108, 568, 203, 593), selector light, 508 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K24" authorId="1" shapeId="0">
+    <comment ref="L22" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground: ST-07_01.jpg, pixel box (205, 547, 228, 589), selector median, 966 selected pixels.
+Chest panel / collar: ST-07_01.jpg, pixel box (205, 399, 228, 441), selector median, 966 selected pixels.
+Fine panel borders: ST-07_01.jpg, pixel box (117, 482, 226, 498), selector dark, 349 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K25" authorId="1" shapeId="0">
+    <comment ref="L23" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground: ST-07_02.jpg, pixel box (204, 547, 228, 589), selector median, 1008 selected pixels.
+Chest panel / collar: ST-07_02.jpg, pixel box (204, 399, 228, 441), selector median, 1008 selected pixels.
+Fine panel borders: ST-07_02.jpg, pixel box (162, 339, 271, 360), selector red, 694 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K26" authorId="1" shapeId="0">
+    <comment ref="L24" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-09_01.jpg, pixel box (223, 463, 251, 504), selector median, 1148 selected pixels.
+Collar / cuff tipping: ST-09_01.jpg, pixel box (57, 470, 90, 486), selector light, 106 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K27" authorId="1" shapeId="0">
+    <comment ref="L25" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-09_02.jpg, pixel box (224, 463, 251, 504), selector median, 1107 selected pixels.
+Collar / cuff tipping: ST-09_02.jpg, pixel box (58, 470, 90, 486), selector light, 103 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K28" authorId="1" shapeId="0">
+    <comment ref="L26" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / neck / rib trim: ST-10_01.jpg, pixel box (127, 309, 255, 469), selector light, 4097 selected pixels.
+Horizontal stripes: ST-10_01.jpg, pixel box (127, 309, 255, 469), selector dark, 4097 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K29" authorId="1" shapeId="0">
+    <comment ref="L27" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / neck / rib trim: ST-10_02.jpg, pixel box (127, 309, 255, 469), selector light, 4096 selected pixels.
+Horizontal stripes: ST-10_02.jpg, pixel box (127, 309, 255, 469), selector dark, 4099 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K30" authorId="1" shapeId="0">
+    <comment ref="L28" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / neck / rib trim: ST-10_03.jpg, pixel box (127, 309, 255, 469), selector light, 4176 selected pixels.
+Horizontal stripes: ST-10_03.jpg, pixel box (127, 309, 255, 469), selector dark, 4101 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K31" authorId="1" shapeId="0">
+    <comment ref="L29" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Mesh ground: ST-11_01.jpg, pixel box (134, 469, 227, 597), selector light, 2467 selected pixels.
+Neck / shoulder stripes / back graphic: ST-11_01_detail.jpg, pixel box (122, 361, 169, 434), selector red, 3205 selected pixels.
+Badge dark details: ST-11_01_detail.jpg, pixel box (500, 238, 539, 303), selector dark, 509 selected pixels.
+Badge light details: ST-11_01_detail.jpg, pixel box (240, 318, 295, 382), selector light, 729 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K32" authorId="1" shapeId="0">
+    <comment ref="L30" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / collar / rib trim: ST-12_01.jpg, pixel box (146, 431, 169, 473), selector median, 966 selected pixels.
+Vertical pinstripes: ST-12_01.jpg, pixel box (112, 386, 338, 518), selector ink-dark, 299 selected pixels.
+Light vertical pinstripes: ST-12_01.jpg, pixel box (172, 402, 178, 502), selector light, 122 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K33" authorId="1" shapeId="0">
+    <comment ref="E31" authorId="2" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>Light-blue vertical pinstripes are also visible in the supplied final render, so they are included in the colour list and image-based Pantone comparison.</t>
       </text>
     </comment>
-    <comment ref="K34" authorId="1" shapeId="0">
+    <comment ref="L31" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / collar / rib trim: ST-12_02.jpg, pixel box (227, 447, 250, 490), selector median, 989 selected pixels.
+Primary vertical pinstripes: ST-12_02.jpg, pixel box (67, 378, 176, 510), selector blue-dark, 77 selected pixels.
+Secondary vertical pinstripes: ST-12_02.jpg, pixel box (218, 411, 232, 510), selector red, 350 selected pixels.
+Light-blue vertical pinstripes: ST-12_02.jpg, pixel box (165, 386, 182, 502), selector blue, 460 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K35" authorId="1" shapeId="0">
+    <comment ref="L32" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-13_01.jpg, pixel box (195, 367, 223, 403), selector median, 1008 selected pixels.
+Collar / zip trim / tipping / stag: ST-13_01.jpg, pixel box (257, 124, 279, 189), selector dark, 287 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K36" authorId="1" shapeId="0">
+    <comment ref="L33" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body: ST-13_02.jpg, pixel box (196, 369, 224, 406), selector median, 1036 selected pixels.
+Collar / zip trim / tipping / stag: ST-13_02.jpg, pixel box (258, 125, 281, 191), selector dark, 305 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K37" authorId="1" shapeId="0">
+    <comment ref="L34" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / collar / cuffs: ST-14_01.jpg, pixel box (224, 577, 291, 644), selector light, 994 selected pixels.
+Broad chest band: ST-14_01.jpg, pixel box (208, 424, 285, 450), selector dark, 581 selected pixels.
+Fine stripe borders: ST-14_01.jpg, pixel box (175, 386, 285, 400), selector blue, 221 selected pixels.
+Badge / zip-pull accent: ST-14_01.jpg, pixel box (364, 400, 403, 442), selector red, 422 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K38" authorId="1" shapeId="0">
+    <comment ref="L35" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / collar / cuffs: ST-14_02.jpg, pixel box (205, 578, 266, 646), selector dark, 854 selected pixels.
+Broad chest band: ST-14_02.jpg, pixel box (190, 450, 261, 476), selector light, 381 selected pixels.
+Fine stripe borders: ST-14_02.jpg, pixel box (159, 401, 261, 416), selector red, 824 selected pixels.
+Badge / zip-pull accent: ST-14_02.jpg, pixel box (339, 422, 366, 446), selector red, 588 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K39" authorId="1" shapeId="0">
+    <comment ref="L36" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / collar / placket: ST-15_01.jpg, pixel box (137, 389, 152, 423), selector median, 510 selected pixels.
+Broad stripes: ST-15_01.jpg, pixel box (137, 462, 152, 496), selector median, 510 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K40" authorId="1" shapeId="0">
+    <comment ref="L37" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground: ST-15_02.jpg, pixel box (136, 415, 152, 449), selector median, 544 selected pixels.
+Collar / broad stripes: ST-15_02.jpg, pixel box (136, 342, 152, 376), selector median, 544 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K41" authorId="1" shapeId="0">
+    <comment ref="L38" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / collar / rib trim: ST-16_01.jpg, pixel box (170, 273, 311, 330), selector light, 1608 selected pixels.
+Fine stripes / emblem: ST-16_01.jpg, pixel box (170, 273, 311, 330), selector dark, 1608 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K42" authorId="1" shapeId="0">
+    <comment ref="L39" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / collar: ST-16_02.jpg, pixel box (164, 273, 301, 330), selector dark, 1562 selected pixels.
+Fine stripes / rib trim: ST-16_02.jpg, pixel box (164, 273, 301, 330), selector light, 1562 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K43" authorId="1" shapeId="0">
+    <comment ref="L40" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-17_01.jpg, pixel box (180, 461, 204, 500), selector median, 936 selected pixels.
+Embroidery petals: ST-17_01.jpg, pixel box (295, 290, 365, 376), selector light, 1231 selected pixels.
+Embroidery leaves: ST-17_01.jpg, pixel box (299, 399, 342, 454), selector green, 682 selected pixels.
+Embroidery stems / outlines: ST-17_01.jpg, pixel box (299, 368, 342, 423), selector dark, 473 selected pixels.
+Flower centres / bee yellow: ST-17_01.jpg, pixel box (258, 375, 291, 415), selector yellow, 23 selected pixels.
+Bee dark details: ST-17_01.jpg, pixel box (258, 375, 291, 415), selector dark, 264 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K44" authorId="1" shapeId="0">
+    <comment ref="L41" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-17_02.jpg, pixel box (169, 445, 193, 484), selector median, 936 selected pixels.
+Embroidery petals / light outlines: ST-17_02_detail.jpg, pixel box (104, 28, 144, 65), selector light, 296 selected pixels.
+Embroidery leaves: ST-17_02_detail.jpg, pixel box (121, 136, 153, 173), selector green, 454 selected pixels.
+Flower centres / bee yellow: ST-17_02_detail.jpg, pixel box (28, 119, 75, 153), selector yellow, 150 selected pixels.
+Bee dark details: ST-17_02_detail.jpg, pixel box (33, 136, 70, 157), selector dark, 157 selected pixels.</t>
       </text>
     </comment>
-    <comment ref="K45" authorId="1" shapeId="0">
+    <comment ref="L42" authorId="1" shapeId="0">
       <text>
-        <t>PANTONE FHI TCX textile references. [PDF] = code printed in supplied final PDF and number/name located in the checked third-party TCX dataset; it does not certify physical colour accuracy. [PROPOSED] = suggested design reference from screen appearance, NOT an exact measured match or production-approved shade. Display colour names may differ from reference-library names. Every reference needs physical TCX swatch and yarn/lab-dip approval. Dataset: pantone-tcx 2.2.4, ISC, https://github.com/pedroduke/pantone-tcx. It is not an official Pantone approval source.</t>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-18_01.jpg, pixel box (213, 431, 237, 473), selector median, 1008 selected pixels.
+Collar / cuff / hem tipping: ST-18_01.jpg, pixel box (144, 649, 307, 683), selector light, 1109 selected pixels.</t>
+      </text>
+    </comment>
+    <comment ref="L43" authorId="1" shapeId="0">
+      <text>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Body / collar: ST-18_02.jpg, pixel box (214, 431, 237, 473), selector median, 966 selected pixels.
+Collar / cuff / hem tipping: ST-18_02.jpg, pixel box (144, 675, 307, 706), selector dark, 1011 selected pixels.</t>
+      </text>
+    </comment>
+    <comment ref="L44" authorId="1" shapeId="0">
+      <text>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / neck / rib trim: ST-19_01.jpg, pixel box (94, 236, 179, 343), selector light, 1823 selected pixels.
+Warm micro stripes: ST-19_01.jpg, pixel box (94, 236, 179, 343), selector warm, 6618 selected pixels.
+Cool micro stripes: ST-19_01.jpg, pixel box (94, 236, 179, 343), selector neutral, 5400 selected pixels.</t>
+      </text>
+    </comment>
+    <comment ref="L45" authorId="1" shapeId="0">
+      <text>
+        <t>APPROXIMATE DIGITAL IMAGE MATCHES ONLY. Fabric regions were sampled from the supplied final render images and compared to the pantone-tcx 2.2.4 third-party RGB dataset using CIELAB D65 / CIEDE2000. Numbers describe closest listed SCREEN RGB references, not measured physical yarn colours. No white-balance calibration is possible from these images. Lighting, compression, tiny stripe/embroidery pixels and the dataset limit accuracy. Different renders bearing the same generic colour name may have different digital matches. Screen deltaE00 is a numeric comparison of two RGB swatches, not a physical colour tolerance. Validate every shade on a physical Pantone FHI TCX cotton chip and actual yarn lab dip. Original PDF code labels are preserved in the separate CSV for comparison, not accepted as automatically correct.
+Sample audit:
+Ground / neck / rib trim: ST-19_02.jpg, pixel box (79, 217, 164, 310), selector red, 7896 selected pixels.
+Warm micro stripes: ST-19_02_detail.jpg, pixel box (28, 108, 100, 155), selector light, 678 selected pixels.
+Cool micro stripes: ST-19_02_detail.jpg, pixel box (21, 96, 107, 174), selector gray-light, 156 selected pixels.</t>
       </text>
     </comment>
   </commentList>
@@ -1726,6 +1898,2206 @@
         <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId57"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId58"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId59"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId60"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId61"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId62"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId63"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId64"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId65"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId66"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId67"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="68" name="Image 68" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId68"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="69" name="Image 69" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId69"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="70" name="Image 70" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId70"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="71" name="Image 71" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId71"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="72" name="Image 72" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId72"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="73" name="Image 73" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId73"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="74" name="Image 74" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId74"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="75" name="Image 75" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId75"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="76" name="Image 76" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId76"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="77" name="Image 77" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId77"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="78" name="Image 78" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId78"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="79" name="Image 79" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId79"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="80" name="Image 80" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId80"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="81" name="Image 81" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId81"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="82" name="Image 82" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId82"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="83" name="Image 83" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId83"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="84" name="Image 84" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId84"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="85" name="Image 85" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId85"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="86" name="Image 86" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId86"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="87" name="Image 87" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId87"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="88" name="Image 88" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId88"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="89" name="Image 89" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId89"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="90" name="Image 90" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId90"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="91" name="Image 91" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId91"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="92" name="Image 92" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId92"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="93" name="Image 93" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId93"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="94" name="Image 94" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId94"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="95" name="Image 95" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId95"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="96" name="Image 96" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId96"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="97" name="Image 97" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId97"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="98" name="Image 98" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId98"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="99" name="Image 99" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId99"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="100" name="Image 100" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId100"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="101" name="Image 101" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId101"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="102" name="Image 102" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId102"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="103" name="Image 103" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId103"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="104" name="Image 104" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId104"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="105" name="Image 105" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId105"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="106" name="Image 106" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId106"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="107" name="Image 107" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId107"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="108" name="Image 108" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId108"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="109" name="Image 109" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId109"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="110" name="Image 110" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId110"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="111" name="Image 111" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId111"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="112" name="Image 112" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId112"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="113" name="Image 113" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId113"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="114" name="Image 114" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId114"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="115" name="Image 115" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId115"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="116" name="Image 116" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId116"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="117" name="Image 117" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId117"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="118" name="Image 118" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId118"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="119" name="Image 119" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId119"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="120" name="Image 120" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId120"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="4076700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="121" name="Image 121" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId121"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="4076700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="122" name="Image 122" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId122"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="123" name="Image 123" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId123"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="124" name="Image 124" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId124"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="125" name="Image 125" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId125"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="126" name="Image 126" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId126"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="127" name="Image 127" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId127"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="128" name="Image 128" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId128"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="129" name="Image 129" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId129"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="130" name="Image 130" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId130"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="131" name="Image 131" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId131"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2476500" cy="2333625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="132" name="Image 132" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId132"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1916,7 +4288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1929,7 +4301,9 @@
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="100" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="104" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1985,7 +4359,17 @@
       </c>
       <c r="K1" s="8" t="inlineStr">
         <is>
-          <t>Pantone TCX Reference</t>
+          <t>Sampled Image Colours</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>Closest Pantone TCX — APPROXIMATE</t>
+        </is>
+      </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>Pantone Screen Swatches</t>
         </is>
       </c>
     </row>
@@ -2034,11 +4418,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K2" s="14" t="inlineStr">
-        <is>
-          <t>Body / collar — Dark Olive: 19-0323 TCX (Chive) [PROPOSED]
-Side panel / contrast sleeve — Off White: 11-0602 TCX (Snow White) [PROPOSED]
-Cable stripe — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]</t>
+      <c r="L2" s="17" t="inlineStr">
+        <is>
+          <t>Body / collar — Dark Olive: 19-0509 TCX (Rosin)
+Image #2A2C21 → reference #36362D | screen ΔE00 3.85 [APPROX.]
+Side panel / contrast sleeve — Off White: 12-0601 TCX (Eggnog)
+Image #EADECE → reference #ECE1D3 | screen ΔE00 1.04 [APPROX.]
+Cable stripe — Burgundy: 19-1317 TCX (Bitter Chocolate)
+Image #3F1C19 → reference #503130 | screen ΔE00 6.64 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2087,11 +4474,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K3" s="15" t="inlineStr">
-        <is>
-          <t>Body / collar — Denim Blue: 17-4021 TCX (Faded Denim) [PROPOSED]
-Side panel / contrast sleeve — Off White: 11-0602 TCX (Snow White) [PROPOSED]
-Cable stripe — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+      <c r="L3" s="18" t="inlineStr">
+        <is>
+          <t>Body / collar — Denim Blue: 18-3922 TCX (Coronet Blue)
+Image #556F90 → reference #59728E | screen ΔE00 1.96 [APPROX.]
+Side panel / contrast sleeve — Off White: 12-5202 TCX (Turtledove)
+Image #E4DBCC → reference #DED7C8 | screen ΔE00 1.42 [APPROX.]
+Cable stripe — Navy: 19-3831 TCX (Maritime Blue)
+Image #1C253D → reference #27293D | screen ΔE00 3.29 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2140,9 +4530,10 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>Body / collar / rib trim — Classic Beige: 15-1217 TCX (Mojave Desert) [PDF]</t>
+      <c r="L4" s="17" t="inlineStr">
+        <is>
+          <t>Body / collar / rib trim — Classic Beige: 16-1310 TCX (Natural)
+Image #AB9077 → reference #AA907D | screen ΔE00 2.39 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2191,9 +4582,10 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K5" s="15" t="inlineStr">
-        <is>
-          <t>Body / collar / rib trim — Grounded Green: 19-0323 TCX (Chive) [PDF]</t>
+      <c r="L5" s="18" t="inlineStr">
+        <is>
+          <t>Body / collar / rib trim — Grounded Green: 19-0509 TCX (Rosin)
+Image #393728 → reference #36362D | screen ΔE00 3.07 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2242,10 +4634,12 @@
           <t>Relaxed Fit</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>Ground — Classic Beige: 15-1217 TCX (Mojave Desert) [PDF]
-Floral motif — Bright White: 11-0601 TCX (Bright White) [PDF]</t>
+      <c r="L6" s="17" t="inlineStr">
+        <is>
+          <t>Ground — Classic Beige: 12-1404 TCX (Pink Tint)
+Image #DAC7B6 → reference #DBCBBD | screen ΔE00 1.66 [APPROX.]
+Floral motif — Bright White: 12-1108 TCX (Dew)
+Image #ECDCCD → reference #EEDED1 | screen ΔE00 1.04 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2294,11 +4688,12 @@
           <t>Relaxed Fit</t>
         </is>
       </c>
-      <c r="K7" s="16" t="inlineStr">
-        <is>
-          <t>Ground — Eucalyptus: 16-0110 TCX (Desert Sage) [PROPOSED]
-Floral motif — Natural Cotton: 11-0602 TCX (Snow White) [PDF]
-SOURCE-CODE CHECK REQUIRED — see cell comment.</t>
+      <c r="L7" s="18" t="inlineStr">
+        <is>
+          <t>Ground — Eucalyptus: 18-0312 TCX (Deep Lichen Green)
+Image #6C6B57 → reference #6E6E5C | screen ΔE00 1.45 [APPROX.]
+Floral motif — Natural Cotton: 16-0213 TCX (Tea)
+Image #909078 → reference #999B85 | screen ΔE00 3.72 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2347,11 +4742,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K8" s="16" t="inlineStr">
-        <is>
-          <t>Body / collar — Earthy Brown: 18-1222 TCX (Cocoa Brown) [PROPOSED]
-Collar / placket / cuff piping — Natural Cotton: 11-0602 TCX (Snow White) [PDF]
-SOURCE-CODE CHECK REQUIRED — see cell comment.</t>
+      <c r="L8" s="17" t="inlineStr">
+        <is>
+          <t>Body / collar — Earthy Brown: 19-1435 TCX (Cherry Mahogany)
+Image #683C30 → reference #66352B | screen ΔE00 2.42 [APPROX.]
+Collar / placket / cuff piping — Natural Cotton: 11-1302 TCX (Sea Salt)
+Image #F4E7DE → reference #F1E6DE | screen ΔE00 0.88 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2400,10 +4796,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K9" s="15" t="inlineStr">
-        <is>
-          <t>Body / collar — Classic Navy: 19-4029 TCX (Navy Peony) [PDF]
-Collar / placket / cuff piping — Natural Cotton: 11-0602 TCX (Snow White) [PDF]</t>
+      <c r="L9" s="18" t="inlineStr">
+        <is>
+          <t>Body / collar — Classic Navy: 19-3831 TCX (Maritime Blue)
+Image #1D2339 → reference #27293D | screen ΔE00 2.66 [APPROX.]
+Collar / placket / cuff piping — Natural Cotton: 11-4202 TCX (Star White)
+Image #ECEDE6 → reference #EFEFE8 | screen ΔE00 0.67 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2452,10 +4850,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K10" s="14" t="inlineStr">
-        <is>
-          <t>Body — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Collar / placket stripes — Chocolate Brown: 19-0912 TCX (Chocolate Brown) [PROPOSED]</t>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t>Body — Natural Cotton: 12-0605 TCX (Angora)
+Image #DCD1BE → reference #DFD1BB | screen ΔE00 1.43 [APPROX.]
+Collar / placket stripes — Chocolate Brown: 19-0712 TCX (Demitasse)
+Image #3C2615 → reference #40342B | screen ΔE00 7.10 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2504,10 +4904,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K11" s="15" t="inlineStr">
-        <is>
-          <t>Body — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]
-Collar / placket stripes — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L11" s="18" t="inlineStr">
+        <is>
+          <t>Body — Burgundy: 19-1531 TCX (Sun Dried Tomato)
+Image #731B24 → reference #752329 | screen ΔE00 1.55 [APPROX.]
+Collar / placket stripes — Natural Cotton: 11-0105 TCX (Antique White)
+Image #ECE1D1 → reference #EDE3D2 | screen ΔE00 0.85 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2556,9 +4958,10 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>Body / neck / cuffs / hem — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Natural Cotton: 13-0905 TCX (Birch)
+Image #E1D9CE → reference #DDD5C7 | screen ΔE00 1.68 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2607,9 +5010,10 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K13" s="15" t="inlineStr">
-        <is>
-          <t>Body / neck / cuffs / hem — Black: 19-0303 TCX (Jet Black) [PROPOSED]</t>
+      <c r="L13" s="18" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Black: 19-3911 TCX (Black Beauty)
+Image #201F24 → reference #26262A | screen ΔE00 2.39 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2658,9 +5062,10 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>Body / neck / cuffs / hem — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+      <c r="L14" s="17" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Navy: 19-3831 TCX (Maritime Blue)
+Image #24263B → reference #27293D | screen ΔE00 1.07 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2709,9 +5114,10 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K15" s="15" t="inlineStr">
-        <is>
-          <t>Body / neck / cuffs / hem — Sage Green: 16-0110 TCX (Desert Sage) [PROPOSED]</t>
+      <c r="L15" s="18" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Sage Green: 17-0115 TCX (Oil Green)
+Image #7C8373 → reference #80856D | screen ΔE00 3.21 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2760,9 +5166,10 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K16" s="14" t="inlineStr">
-        <is>
-          <t>Body / neck / cuffs / hem — Powder Blue: 14-4214 TCX (Powder Blue) [PROPOSED]</t>
+      <c r="L16" s="17" t="inlineStr">
+        <is>
+          <t>Body / neck / cuffs / hem — Powder Blue: 15-4008 TCX (Blue Fog)
+Image #9AA9BC → reference #9BABBB | screen ΔE00 1.66 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2811,10 +5218,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K17" s="15" t="inlineStr">
-        <is>
-          <t>Body — Powder Blue: 14-4214 TCX (Powder Blue) [PROPOSED]
-Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L17" s="18" t="inlineStr">
+        <is>
+          <t>Body — Powder Blue: 15-4008 TCX (Blue Fog)
+Image #A4ACB7 → reference #9BABBB | screen ΔE00 3.19 [APPROX.]
+Collar / placket / cuffs / hem — Off White: 11-0606 TCX (Pristine)
+Image #F1E8D8 → reference #F2E8DA | screen ΔE00 1.15 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2863,10 +5272,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K18" s="14" t="inlineStr">
-        <is>
-          <t>Body — Dusty Rose: 14-1506 TCX (Rose Smoke) [PROPOSED]
-Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L18" s="17" t="inlineStr">
+        <is>
+          <t>Body — Dusty Rose: 14-1309 TCX (Peach Whip)
+Image #DABDB5 → reference #DBBEB7 | screen ΔE00 0.54 [APPROX.]
+Collar / placket / cuffs / hem — Off White: 11-0606 TCX (Pristine)
+Image #F2E8D9 → reference #F2E8DA | screen ΔE00 0.44 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2915,10 +5326,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K19" s="15" t="inlineStr">
-        <is>
-          <t>Body — Sage Green: 16-0110 TCX (Desert Sage) [PROPOSED]
-Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L19" s="18" t="inlineStr">
+        <is>
+          <t>Body — Sage Green: 17-0115 TCX (Oil Green)
+Image #8B8B73 → reference #80856D | screen ΔE00 3.43 [APPROX.]
+Collar / placket / cuffs / hem — Off White: 11-0105 TCX (Antique White)
+Image #F0E7D7 → reference #EDE3D2 | screen ΔE00 0.98 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -2967,10 +5380,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K20" s="14" t="inlineStr">
-        <is>
-          <t>Body — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
-Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L20" s="17" t="inlineStr">
+        <is>
+          <t>Body — Navy: 19-4024 TCX (Dress Blues)
+Image #2C3346 → reference #2A3244 | screen ΔE00 0.91 [APPROX.]
+Collar / placket / cuffs / hem — Off White: 11-0105 TCX (Antique White)
+Image #EFE6D6 → reference #EDE3D2 | screen ΔE00 0.80 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3019,10 +5434,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K21" s="15" t="inlineStr">
-        <is>
-          <t>Body — Oatmeal: 13-0401 TCX (Oatmeal) [PROPOSED]
-Collar / placket / cuffs / hem — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L21" s="18" t="inlineStr">
+        <is>
+          <t>Body — Oatmeal: 13-1012 TCX (Frosted Almond)
+Image #CFC0AE → reference #D2C2AC | screen ΔE00 1.58 [APPROX.]
+Collar / placket / cuffs / hem — Off White: 11-0104 TCX (Vanilla Ice)
+Image #F2EADA → reference #F0EADA | screen ΔE00 0.98 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3071,11 +5488,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K22" s="14" t="inlineStr">
-        <is>
-          <t>Ground — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Chest panel / collar — Denim Blue: 17-4021 TCX (Faded Denim) [PROPOSED]
-Fine panel borders — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+      <c r="L22" s="17" t="inlineStr">
+        <is>
+          <t>Ground — Natural Cotton: 11-0701 TCX (Whisper White)
+Image #EFE7DC → reference #EDE6DB | screen ΔE00 0.56 [APPROX.]
+Chest panel / collar — Denim Blue: 16-3929 TCX (Grapemist)
+Image #7D92BD → reference #8398CA | screen ΔE00 2.50 [APPROX.]
+Fine panel borders — Navy: 19-3831 TCX (Maritime Blue)
+Image #09152D → reference #27293D | screen ΔE00 7.32 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3124,11 +5544,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K23" s="15" t="inlineStr">
-        <is>
-          <t>Ground — Butter Yellow: 13-0822 TCX (Sunlight) [PROPOSED]
-Chest panel / collar — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Fine panel borders — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]</t>
+      <c r="L23" s="18" t="inlineStr">
+        <is>
+          <t>Ground — Butter Yellow: 13-0815 TCX (Banana Crepe)
+Image #E3D1AE → reference #E7D3AD | screen ΔE00 1.08 [APPROX.]
+Chest panel / collar — Natural Cotton: 11-0104 TCX (Vanilla Ice)
+Image #F2EBDB → reference #F0EADA | screen ΔE00 0.55 [APPROX.]
+Fine panel borders — Burgundy: 19-1724 TCX (Cabernet)
+Image #511419 → reference #64242E | screen ΔE00 5.85 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3177,10 +5600,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>Body / collar — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
-Collar / cuff tipping — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L24" s="17" t="inlineStr">
+        <is>
+          <t>Body / collar — Navy: 19-3831 TCX (Maritime Blue)
+Image #242A3E → reference #27293D | screen ΔE00 1.94 [APPROX.]
+Collar / cuff tipping — Off White: 11-0907 TCX (Pearled Ivory)
+Image #F1E0CC → reference #F0DFCC | screen ΔE00 0.46 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3229,10 +5654,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K25" s="15" t="inlineStr">
-        <is>
-          <t>Body / collar — Rust: 18-1248 TCX (Rust) [PROPOSED]
-Collar / cuff tipping — Off White: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L25" s="18" t="inlineStr">
+        <is>
+          <t>Body / collar — Rust: 19-1250 TCX (Picante)
+Image #833622 → reference #8D3F2D | screen ΔE00 3.18 [APPROX.]
+Collar / cuff tipping — Off White: 11-0809 TCX (Ecru)
+Image #F6DFC5 → reference #F3DFCA | screen ΔE00 1.75 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3281,10 +5708,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K26" s="14" t="inlineStr">
-        <is>
-          <t>Ground / neck / rib trim — Off White: 11-0602 TCX (Snow White) [PROPOSED]
-Horizontal stripes — Denim Blue: 17-4021 TCX (Faded Denim) [PROPOSED]</t>
+      <c r="L26" s="17" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Off White: 11-0607 TCX (Sugar Swizzle)
+Image #F1EDE6 → reference #F3EEE7 | screen ΔE00 0.56 [APPROX.]
+Horizontal stripes — Denim Blue: 18-4025 TCX (Copen Blue)
+Image #536E89 → reference #516B84 | screen ΔE00 1.32 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3333,10 +5762,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K27" s="15" t="inlineStr">
-        <is>
-          <t>Ground / neck / rib trim — Off White: 11-0602 TCX (Snow White) [PROPOSED]
-Horizontal stripes — Rust: 18-1248 TCX (Rust) [PROPOSED]</t>
+      <c r="L27" s="18" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Off White: 12-0601 TCX (Eggnog)
+Image #F0E4D5 → reference #ECE1D3 | screen ΔE00 0.84 [APPROX.]
+Horizontal stripes — Rust: 17-1143 TCX (Hazel)
+Image #B36D46 → reference #AE7250 | screen ΔE00 2.46 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3385,10 +5816,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K28" s="14" t="inlineStr">
-        <is>
-          <t>Ground / neck / rib trim — Off White: 11-0602 TCX (Snow White) [PROPOSED]
-Horizontal stripes — Olive Green: 18-0622 TCX (Olive Drab) [PROPOSED]</t>
+      <c r="L28" s="17" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Off White: 13-1006 TCX (Creme Brulee)
+Image #DCCEB8 → reference #DBCCB5 | screen ΔE00 0.65 [APPROX.]
+Horizontal stripes — Olive Green: 18-0521 TCX (Burnt Olive)
+Image #696348 → reference #646049 | screen ΔE00 1.99 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3437,12 +5870,16 @@
           <t>Relaxed Fit</t>
         </is>
       </c>
-      <c r="K29" s="15" t="inlineStr">
-        <is>
-          <t>Mesh ground — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Neck / shoulder stripes / back graphic — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]
-Badge dark details — Charcoal: 19-4007 TCX (Anthracite) [PROPOSED]
-Badge light details — White: 11-0601 TCX (Bright White) [PROPOSED]</t>
+      <c r="L29" s="18" t="inlineStr">
+        <is>
+          <t>Mesh ground — Natural Cotton: 13-1405 TCX (Shell)
+Image #E0D0C8 → reference #E1CFC6 | screen ΔE00 0.81 [APPROX.]
+Neck / shoulder stripes / back graphic — Burgundy: 19-1726 TCX (Cordovan)
+Image #6E3138 → reference #702F3B | screen ΔE00 1.80 [APPROX.]
+Badge dark details — Charcoal: 19-4008 TCX (Meteorite)
+Image #16120D → reference #2B2929 | screen ΔE00 7.51 [APPROX.]
+Badge light details — White: 11-4800 TCX (Blanc De Blanc)
+Image #EFEFEF → reference #E7E9E7 | screen ΔE00 2.16 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3491,10 +5928,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K30" s="14" t="inlineStr">
-        <is>
-          <t>Ground / collar / rib trim — Powder Blue: 14-4214 TCX (Powder Blue) [PROPOSED]
-Vertical pinstripes — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+      <c r="L30" s="17" t="inlineStr">
+        <is>
+          <t>Ground / collar / rib trim — Powder Blue: 13-3920 TCX (Halogen Blue)
+Image #C9D1E4 → reference #BDC6DC | screen ΔE00 2.92 [APPROX.]
+Vertical pinstripes — Navy: 19-4024 TCX (Dress Blues)
+Image #253348 → reference #2A3244 | screen ΔE00 2.26 [APPROX.]
+Light vertical pinstripes — White: 11-4601 TCX (Bit Of Blue)
+Image #F4FBFE → reference #E2EAEB | screen ΔE00 3.83 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3521,7 +5962,7 @@
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>White / Navy / Burgundy</t>
+          <t>White / Navy / Burgundy / Powder Blue</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
@@ -3543,11 +5984,16 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K31" s="15" t="inlineStr">
-        <is>
-          <t>Ground / collar / rib trim — White: 11-0601 TCX (Bright White) [PROPOSED]
-Primary vertical pinstripes — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
-Secondary vertical pinstripes — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]</t>
+      <c r="L31" s="18" t="inlineStr">
+        <is>
+          <t>Ground / collar / rib trim — White: 11-1001 TCX (White Alyssum)
+Image #F1F0F1 → reference #EFEBE7 | screen ΔE00 2.84 [APPROX.]
+Primary vertical pinstripes — Navy: 19-3731 TCX (Parachute Purple)
+Image #18163D → reference #392852 | screen ΔE00 7.60 [APPROX.]
+Secondary vertical pinstripes — Burgundy: 17-1623 TCX (Rose Wine)
+Image #AB5268 → reference #A4596D | screen ΔE00 2.54 [APPROX.]
+Light-blue vertical pinstripes — Powder Blue: 15-3919 TCX (Serenity)
+Image #91A4C3 → reference #91A8D0 | screen ΔE00 2.66 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3596,10 +6042,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K32" s="14" t="inlineStr">
-        <is>
-          <t>Body — Deep Teal: 19-4914 TCX (Deep Teal) [PROPOSED]
-Collar / zip trim / tipping / stag — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+      <c r="L32" s="17" t="inlineStr">
+        <is>
+          <t>Body — Deep Teal: 19-4517 TCX (Mediterranea)
+Image #2B5860 → reference #32575D | screen ΔE00 1.53 [APPROX.]
+Collar / zip trim / tipping / stag — Navy: 19-3911 TCX (Black Beauty)
+Image #090C17 → reference #26262A | screen ΔE00 8.02 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3648,10 +6096,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K33" s="15" t="inlineStr">
-        <is>
-          <t>Body — Sage Green: 16-0110 TCX (Desert Sage) [PROPOSED]
-Collar / zip trim / tipping / stag — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]</t>
+      <c r="L33" s="18" t="inlineStr">
+        <is>
+          <t>Body — Sage Green: 15-5706 TCX (Frosty Green)
+Image #9DB3A6 → reference #A3B5A6 | screen ΔE00 1.73 [APPROX.]
+Collar / zip trim / tipping / stag — Navy: 19-3911 TCX (Black Beauty)
+Image #0E1217 → reference #26262A | screen ΔE00 6.62 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3700,12 +6150,16 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K34" s="14" t="inlineStr">
-        <is>
-          <t>Ground / collar / cuffs — White: 11-0601 TCX (Bright White) [PROPOSED]
-Broad chest band — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
-Fine stripe borders — Powder Blue: 14-4214 TCX (Powder Blue) [PROPOSED]
-Badge / zip-pull accent — Red: 18-1664 TCX (Fiery Red) [PROPOSED]</t>
+      <c r="L34" s="17" t="inlineStr">
+        <is>
+          <t>Ground / collar / cuffs — White: 11-1001 TCX (White Alyssum)
+Image #FDF6F4 → reference #EFEBE7 | screen ΔE00 3.17 [APPROX.]
+Broad chest band — Navy: 19-3933 TCX (Medieval Blue)
+Image #1C2542 → reference #29304E | screen ΔE00 3.60 [APPROX.]
+Fine stripe borders — Powder Blue: 13-4304 TCX (Ballad Blue)
+Image #C4D1E1 → reference #C0CEDA | screen ΔE00 2.20 [APPROX.]
+Badge / zip-pull accent — Red: 17-1664 TCX (Poppy Red)
+Image #D53E3F → reference #DC343B | screen ΔE00 1.42 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3754,12 +6208,16 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K35" s="15" t="inlineStr">
-        <is>
-          <t>Ground / collar / cuffs — Navy: 19-4029 TCX (Navy Peony) [PROPOSED]
-Broad chest band — Butter Yellow: 13-0822 TCX (Sunlight) [PROPOSED]
-Fine stripe borders — Dusty Pink: 14-1316 TCX (Dusty Pink) [PROPOSED]
-Badge / zip-pull accent — Red: 18-1664 TCX (Fiery Red) [PROPOSED]</t>
+      <c r="L35" s="18" t="inlineStr">
+        <is>
+          <t>Ground / collar / cuffs — Navy: 19-3922 TCX (Sky Captain)
+Image #060C1E → reference #262934 | screen ΔE00 8.80 [APPROX.]
+Broad chest band — Butter Yellow: 13-0932 TCX (Cornsilk)
+Image #F6CE81 → reference #EDC373 | screen ΔE00 2.66 [APPROX.]
+Fine stripe borders — Dusty Pink: 15-1717 TCX (Pink Icing)
+Image #E69EA3 → reference #EEA0A6 | screen ΔE00 1.47 [APPROX.]
+Badge / zip-pull accent — Red: 17-1564 TCX (Fiesta)
+Image #D44236 → reference #DD4132 | screen ΔE00 2.06 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3808,10 +6266,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K36" s="14" t="inlineStr">
-        <is>
-          <t>Ground / collar / placket — Mustard Yellow: 14-0952 TCX (Spicy Mustard) [PROPOSED]
-Broad stripes — Royal Blue: 17-4041 TCX (Marina) [PROPOSED]</t>
+      <c r="L36" s="17" t="inlineStr">
+        <is>
+          <t>Ground / collar / placket — Mustard Yellow: 14-0851 TCX (Samoan Sun)
+Image #F8C454 → reference #FBC85F | screen ΔE00 1.29 [APPROX.]
+Broad stripes — Royal Blue: 16-4032 TCX (Provence)
+Image #6893D7 → reference #658DC6 | screen ΔE00 2.60 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3860,10 +6320,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K37" s="15" t="inlineStr">
-        <is>
-          <t>Ground — Emerald Green: 17-5641 TCX (Emerald) [PROPOSED]
-Collar / broad stripes — Purple: 19-3642 TCX (Royal Purple) [PROPOSED]</t>
+      <c r="L37" s="18" t="inlineStr">
+        <is>
+          <t>Ground — Emerald Green: 18-6018 TCX (Foliage Green)
+Image #376F57 → reference #3E6F58 | screen ΔE00 1.24 [APPROX.]
+Collar / broad stripes — Purple: 19-3750 TCX (Violet Indigo)
+Image #452D61 → reference #3E285C | screen ΔE00 1.79 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3912,10 +6374,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K38" s="14" t="inlineStr">
-        <is>
-          <t>Ground / collar / rib trim — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Fine stripes / emblem — Taupe: 16-1105 TCX (Plaza Taupe) [PROPOSED]</t>
+      <c r="L38" s="17" t="inlineStr">
+        <is>
+          <t>Ground / collar / rib trim — Natural Cotton: 12-0601 TCX (Eggnog)
+Image #EBE0D3 → reference #ECE1D3 | screen ΔE00 0.49 [APPROX.]
+Fine stripes / emblem — Taupe: 16-1336 TCX (Biscuit)
+Image #AE7C5B → reference #B4835B | screen ΔE00 3.27 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -3964,14 +6428,16 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K39" s="15" t="inlineStr">
-        <is>
-          <t>Ground / collar — Royal Blue: 17-4041 TCX (Marina) [PROPOSED]
-Fine stripes / rib trim — White: 11-0601 TCX (Bright White) [PROPOSED]</t>
+      <c r="L39" s="18" t="inlineStr">
+        <is>
+          <t>Ground / collar — Royal Blue: 18-3928 TCX (Dutch Blue)
+Image #4E6591 → reference #4A638D | screen ΔE00 1.16 [APPROX.]
+Fine stripes / rib trim — White: 13-4105 TCX (Lilac Hint)
+Image #D6D8E5 → reference #D0D0DA | screen ΔE00 2.30 [APPROX.]</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="265" customHeight="1">
+    <row r="40" ht="327" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
           <t>ST-17-1</t>
@@ -4016,18 +6482,24 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K40" s="14" t="inlineStr">
-        <is>
-          <t>Body / collar — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Embroidery petals — White: 11-0601 TCX (Bright White) [PROPOSED]
-Embroidery leaves — Olive Green: 18-0622 TCX (Olive Drab) [PROPOSED]
-Embroidery stems / outlines — Chocolate Brown: 19-0912 TCX (Chocolate Brown) [PROPOSED]
-Flower centres / bee yellow — Mustard Yellow: 14-0952 TCX (Spicy Mustard) [PROPOSED]
-Bee dark details — Black: 19-0303 TCX (Jet Black) [PROPOSED]</t>
+      <c r="L40" s="17" t="inlineStr">
+        <is>
+          <t>Body / collar — Natural Cotton: 13-1107 TCX (Whisper Pink)
+Image #DFD2C8 → reference #DACBBE | screen ΔE00 2.11 [APPROX.]
+Embroidery petals — White: 11-1302 TCX (Sea Salt)
+Image #EFE7E2 → reference #F1E6DE | screen ΔE00 1.63 [APPROX.]
+Embroidery leaves — Olive Green: 18-0422 TCX (Loden Green)
+Image #71725A → reference #6E7153 | screen ΔE00 2.41 [APPROX.]
+Embroidery stems / outlines — Chocolate Brown: 19-0419 TCX (Rifle Green)
+Image #44422A → reference #414832 | screen ΔE00 4.99 [APPROX.]
+Flower centres / bee yellow — Mustard Yellow: 16-0726 TCX (Khaki)
+Image #A99D6D → reference #A39264 | screen ΔE00 3.76 [APPROX.]
+Bee dark details — Black: 19-0509 TCX (Rosin)
+Image #393526 → reference #36362D | screen ΔE00 3.60 [APPROX.]</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="245" customHeight="1">
+    <row r="41" ht="276" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
         <is>
           <t>ST-17-2</t>
@@ -4072,13 +6544,18 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K41" s="15" t="inlineStr">
-        <is>
-          <t>Body / collar — Dark Olive: 19-0323 TCX (Chive) [PROPOSED]
-Embroidery petals / light outlines — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Embroidery leaves — Sage Green: 16-0110 TCX (Desert Sage) [PROPOSED]
-Flower centres / bee yellow — Mustard Yellow: 14-0952 TCX (Spicy Mustard) [PROPOSED]
-Bee dark details — Black: 19-0303 TCX (Jet Black) [PROPOSED]</t>
+      <c r="L41" s="18" t="inlineStr">
+        <is>
+          <t>Body / collar — Dark Olive: 19-0516 TCX (Dark Olive)
+Image #48432D → reference #574D35 | screen ΔE00 4.58 [APPROX.]
+Embroidery petals / light outlines — Natural Cotton: 13-0401 TCX (Oatmeal)
+Image #C7C0B2 → reference #CBC3B4 | screen ΔE00 0.96 [APPROX.]
+Embroidery leaves — Sage Green: 19-0419 TCX (Rifle Green)
+Image #414029 → reference #414832 | screen ΔE00 4.71 [APPROX.]
+Flower centres / bee yellow — Mustard Yellow: 17-0929 TCX (Fennel Seed)
+Image #A1895A → reference #998456 | screen ΔE00 2.23 [APPROX.]
+Bee dark details — Black: 19-4008 TCX (Meteorite)
+Image #0D0B06 → reference #2B2929 | screen ΔE00 8.90 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -4127,10 +6604,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K42" s="14" t="inlineStr">
-        <is>
-          <t>Body / collar — Chocolate Brown: 19-0912 TCX (Chocolate Brown) [PROPOSED]
-Collar / cuff / hem tipping — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]</t>
+      <c r="L42" s="17" t="inlineStr">
+        <is>
+          <t>Body / collar — Chocolate Brown: 19-1233 TCX (Tiramisu)
+Image #5E3C2C → reference #634235 | screen ΔE00 2.42 [APPROX.]
+Collar / cuff / hem tipping — Natural Cotton: 11-0606 TCX (Pristine)
+Image #F3EADE → reference #F2E8DA | screen ΔE00 0.93 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -4179,10 +6658,12 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K43" s="15" t="inlineStr">
-        <is>
-          <t>Body / collar — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Collar / cuff / hem tipping — Chocolate Brown: 19-0912 TCX (Chocolate Brown) [PROPOSED]</t>
+      <c r="L43" s="18" t="inlineStr">
+        <is>
+          <t>Body / collar — Natural Cotton: 11-0103 TCX (Egret)
+Image #F1E9DD → reference #F3ECE0 | screen ΔE00 0.77 [APPROX.]
+Collar / cuff / hem tipping — Chocolate Brown: 19-1419 TCX (Chicory Coffee)
+Image #422A1E → reference #4A342E | screen ΔE00 4.57 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -4231,11 +6712,14 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K44" s="14" t="inlineStr">
-        <is>
-          <t>Ground / neck / rib trim — Natural Cotton: 11-0602 TCX (Snow White) [PROPOSED]
-Warm micro stripes — Taupe: 16-1105 TCX (Plaza Taupe) [PROPOSED]
-Cool micro stripes — Grey: 17-4402 TCX (Neutral Gray) [PROPOSED]</t>
+      <c r="L44" s="17" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Natural Cotton: 11-0605 TCX (Jet Stream)
+Image #E8E3DC → reference #EDE6DE | screen ΔE00 1.18 [APPROX.]
+Warm micro stripes — Taupe: 15-4502 TCX (Silver Cloud)
+Image #C4BBB2 → reference #BEB7B0 | screen ΔE00 1.59 [APPROX.]
+Cool micro stripes — Grey: 15-4502 TCX (Silver Cloud)
+Image #BEB6AE → reference #BEB7B0 | screen ΔE00 0.61 [APPROX.]</t>
         </is>
       </c>
     </row>
@@ -4284,16 +6768,19 @@
           <t>Slim Fit</t>
         </is>
       </c>
-      <c r="K45" s="15" t="inlineStr">
-        <is>
-          <t>Ground / neck / rib trim — Burgundy: 19-1617 TCX (Burgundy) [PROPOSED]
-Warm micro stripes — Taupe: 16-1105 TCX (Plaza Taupe) [PROPOSED]
-Cool micro stripes — Grey: 17-4402 TCX (Neutral Gray) [PROPOSED]</t>
+      <c r="L45" s="18" t="inlineStr">
+        <is>
+          <t>Ground / neck / rib trim — Burgundy: 19-1525 TCX (Port)
+Image #6C3236 → reference #663336 | screen ΔE00 1.66 [APPROX.]
+Warm micro stripes — Taupe: 19-1420 TCX (Deep Mahogany)
+Image #543A3B → reference #553B39 | screen ΔE00 1.58 [APPROX.]
+Cool micro stripes — Grey: 18-1409 TCX (Peppercorn)
+Image #715D5B → reference #6C5656 | screen ΔE00 2.74 [APPROX.]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K45"/>
+  <autoFilter ref="A1:M45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>